<commit_message>
-se modifico el codigo para que los excel con los resultados no agreguen lineas vacias en en los proyectos que no tienen datos en sus hojas
</commit_message>
<xml_diff>
--- a/medidor de metricas/automatizacion_completa/metricas_resultados_esp32_android.xlsx
+++ b/medidor de metricas/automatizacion_completa/metricas_resultados_esp32_android.xlsx
@@ -2839,7 +2839,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G5"/>
+  <dimension ref="A1:G3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -2891,25 +2891,47 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>L1-1C2026-AND-M</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr"/>
-      <c r="C2" t="inlineStr"/>
-      <c r="D2" t="inlineStr"/>
-      <c r="E2" t="inlineStr"/>
-      <c r="F2" t="inlineStr"/>
-      <c r="G2" t="inlineStr"/>
+          <t>L1-1C2026-AND-V</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="F2" t="n">
+        <v>2.75</v>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Hay aspectos que requieren observación</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>L1-1C2026-AND-V</t>
+          <t>L2-1C2026-AND-V</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Media</t>
+          <t>Alta</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -2928,57 +2950,9 @@
         </is>
       </c>
       <c r="F3" t="n">
-        <v>2.75</v>
+        <v>3</v>
       </c>
       <c r="G3" t="inlineStr">
-        <is>
-          <t>Hay aspectos que requieren observación</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>L2-1C2026-AND-M</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr"/>
-      <c r="C4" t="inlineStr"/>
-      <c r="D4" t="inlineStr"/>
-      <c r="E4" t="inlineStr"/>
-      <c r="F4" t="inlineStr"/>
-      <c r="G4" t="inlineStr"/>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>L2-1C2026-AND-V</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>Alta</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>Alta</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>Alta</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>Alta</t>
-        </is>
-      </c>
-      <c r="F5" t="n">
-        <v>3</v>
-      </c>
-      <c r="G5" t="inlineStr">
         <is>
           <t>Muy buen uso de concurrencia</t>
         </is>
@@ -2995,7 +2969,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I5"/>
+  <dimension ref="A1:I3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -3059,102 +3033,72 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>L1-1C2026-AND-M</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr"/>
-      <c r="C2" t="inlineStr"/>
-      <c r="D2" t="inlineStr"/>
-      <c r="E2" t="inlineStr"/>
-      <c r="F2" t="inlineStr"/>
-      <c r="G2" t="inlineStr"/>
-      <c r="H2" t="inlineStr"/>
-      <c r="I2" t="inlineStr"/>
+          <t>L1-1C2026-AND-V</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>herramienta modelo</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
+        <v>571</v>
+      </c>
+      <c r="D2" t="n">
+        <v>3</v>
+      </c>
+      <c r="E2" t="n">
+        <v>4024</v>
+      </c>
+      <c r="F2" t="n">
+        <v>141.9</v>
+      </c>
+      <c r="G2" t="n">
+        <v>109.15</v>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>Alto</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>Alto NLOC/token, ajustada por refinamientos.</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>L1-1C2026-AND-V</t>
+          <t>L2-1C2026-AND-V</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>herramienta modelo</t>
+          <t>Context Windows</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>571</v>
+        <v>640</v>
       </c>
       <c r="D3" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E3" t="n">
-        <v>4024</v>
+        <v>107500</v>
       </c>
       <c r="F3" t="n">
-        <v>141.9</v>
+        <v>5.95</v>
       </c>
       <c r="G3" t="n">
-        <v>109.15</v>
+        <v>4.96</v>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Alto</t>
+          <t>Bajo</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
-        <is>
-          <t>Alto NLOC/token, ajustada por refinamientos.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>L2-1C2026-AND-M</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr"/>
-      <c r="C4" t="inlineStr"/>
-      <c r="D4" t="inlineStr"/>
-      <c r="E4" t="inlineStr"/>
-      <c r="F4" t="inlineStr"/>
-      <c r="G4" t="inlineStr"/>
-      <c r="H4" t="inlineStr"/>
-      <c r="I4" t="inlineStr"/>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>L2-1C2026-AND-V</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>Context Windows</t>
-        </is>
-      </c>
-      <c r="C5" t="n">
-        <v>640</v>
-      </c>
-      <c r="D5" t="n">
-        <v>2</v>
-      </c>
-      <c r="E5" t="n">
-        <v>107500</v>
-      </c>
-      <c r="F5" t="n">
-        <v>5.95</v>
-      </c>
-      <c r="G5" t="n">
-        <v>4.96</v>
-      </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>Bajo</t>
-        </is>
-      </c>
-      <c r="I5" t="inlineStr">
         <is>
           <t>Bajo NLOC/token, ajustada por refinamientos.</t>
         </is>

</xml_diff>

<commit_message>
se cambio de logs de error a warnign cuando no existe datos de un proyecto para determinada hoja del excel resultados
</commit_message>
<xml_diff>
--- a/medidor de metricas/automatizacion_completa/metricas_resultados_esp32_android.xlsx
+++ b/medidor de metricas/automatizacion_completa/metricas_resultados_esp32_android.xlsx
@@ -2735,12 +2735,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C5"/>
+  <dimension ref="A1:C1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="18" customWidth="1" min="1" max="1"/>
-    <col width="33" customWidth="1" min="2" max="2"/>
-    <col width="45" customWidth="1" min="3" max="3"/>
+    <col width="9" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="8" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2757,74 +2757,6 @@
       <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Error</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>L1-1C2026-AND-M</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>Smart Mirror</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>Análisis concurrencia: No se encontró el código 'L1-1C2026-AND-M' en Concurrencia</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>L1-1C2026-AND-M</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>Smart Mirror</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>Análisis tokens: No se encontró el código 'L1-1C2026-AND-M' en Datos Tokens</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>L2-1C2026-AND-M</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>Sistema de Atención al Volante</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>Análisis concurrencia: No se encontró el código 'L2-1C2026-AND-M' en Concurrencia</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>L2-1C2026-AND-M</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>Sistema de Atención al Volante</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>Análisis tokens: No se encontró el código 'L2-1C2026-AND-M' en Datos Tokens</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
se agrego la palabra sin datos en la hoja resumen cuando un proyecto no tiene datos en una determinada hoja del excel resultante
</commit_message>
<xml_diff>
--- a/medidor de metricas/automatizacion_completa/metricas_resultados_esp32_android.xlsx
+++ b/medidor de metricas/automatizacion_completa/metricas_resultados_esp32_android.xlsx
@@ -27,11 +27,26 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.00\%"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="4">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <color rgb="00000000"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <b val="1"/>
+      <color rgb="00008000"/>
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
@@ -84,18 +99,22 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -1725,49 +1744,65 @@
           <t>Java</t>
         </is>
       </c>
-      <c r="I2" t="n">
+      <c r="I2" s="4" t="n">
         <v>1.88</v>
       </c>
-      <c r="J2" s="4" t="inlineStr">
+      <c r="J2" s="5" t="inlineStr">
         <is>
           <t>Bajo</t>
         </is>
       </c>
-      <c r="K2" t="n">
+      <c r="K2" s="4" t="n">
         <v>53.1</v>
       </c>
-      <c r="L2" s="4" t="inlineStr">
+      <c r="L2" s="5" t="inlineStr">
         <is>
           <t>Buena</t>
         </is>
       </c>
-      <c r="M2" t="n">
+      <c r="M2" s="4" t="n">
         <v>65.79000000000001</v>
       </c>
-      <c r="N2" t="n">
+      <c r="N2" s="4" t="n">
         <v>2.03</v>
       </c>
-      <c r="O2" s="4" t="inlineStr">
+      <c r="O2" s="5" t="inlineStr">
         <is>
           <t>Predominan issues medios</t>
         </is>
       </c>
-      <c r="P2" t="inlineStr"/>
-      <c r="Q2" s="4" t="inlineStr"/>
-      <c r="R2" t="inlineStr"/>
-      <c r="S2" s="4" t="inlineStr"/>
-      <c r="T2" s="5" t="n">
+      <c r="P2" s="6" t="inlineStr">
+        <is>
+          <t>Sin datos</t>
+        </is>
+      </c>
+      <c r="Q2" s="7" t="inlineStr">
+        <is>
+          <t>Sin datos</t>
+        </is>
+      </c>
+      <c r="R2" s="6" t="inlineStr">
+        <is>
+          <t>Sin datos</t>
+        </is>
+      </c>
+      <c r="S2" s="7" t="inlineStr">
+        <is>
+          <t>Sin datos</t>
+        </is>
+      </c>
+      <c r="T2" s="8" t="n">
         <v>0.125</v>
       </c>
-      <c r="U2" s="4" t="inlineStr">
+      <c r="U2" s="5" t="inlineStr">
         <is>
           <t>Consumo bajo de CPU</t>
         </is>
       </c>
-      <c r="V2" s="5" t="n">
+      <c r="V2" s="8" t="n">
         <v>1.373203285420945</v>
       </c>
-      <c r="W2" s="4" t="inlineStr">
+      <c r="W2" s="5" t="inlineStr">
         <is>
           <t>Consumo bajo de CPU</t>
         </is>
@@ -1814,61 +1849,61 @@
           <t>Java</t>
         </is>
       </c>
-      <c r="I3" t="n">
+      <c r="I3" s="4" t="n">
         <v>1.82</v>
       </c>
-      <c r="J3" s="4" t="inlineStr">
+      <c r="J3" s="5" t="inlineStr">
         <is>
           <t>Bajo</t>
         </is>
       </c>
-      <c r="K3" t="n">
+      <c r="K3" s="4" t="n">
         <v>50.98</v>
       </c>
-      <c r="L3" s="4" t="inlineStr">
+      <c r="L3" s="5" t="inlineStr">
         <is>
           <t>Buena</t>
         </is>
       </c>
-      <c r="M3" t="n">
+      <c r="M3" s="4" t="n">
         <v>15.76</v>
       </c>
-      <c r="N3" t="n">
+      <c r="N3" s="4" t="n">
         <v>2.67</v>
       </c>
-      <c r="O3" s="4" t="inlineStr">
+      <c r="O3" s="5" t="inlineStr">
         <is>
           <t>Presencia de issues altos</t>
         </is>
       </c>
-      <c r="P3" t="n">
+      <c r="P3" s="4" t="n">
         <v>2.75</v>
       </c>
-      <c r="Q3" s="4" t="inlineStr">
+      <c r="Q3" s="5" t="inlineStr">
         <is>
           <t>Hay aspectos que requieren observación</t>
         </is>
       </c>
-      <c r="R3" t="n">
+      <c r="R3" s="4" t="n">
         <v>109.15</v>
       </c>
-      <c r="S3" s="4" t="inlineStr">
+      <c r="S3" s="5" t="inlineStr">
         <is>
           <t>Alto NLOC/token, ajustada por refinamientos.</t>
         </is>
       </c>
-      <c r="T3" s="5" t="n">
+      <c r="T3" s="8" t="n">
         <v>0.125</v>
       </c>
-      <c r="U3" s="4" t="inlineStr">
+      <c r="U3" s="5" t="inlineStr">
         <is>
           <t>Consumo bajo de CPU</t>
         </is>
       </c>
-      <c r="V3" s="5" t="n">
+      <c r="V3" s="8" t="n">
         <v>1.456622176591376</v>
       </c>
-      <c r="W3" s="4" t="inlineStr">
+      <c r="W3" s="5" t="inlineStr">
         <is>
           <t>Consumo bajo de CPU</t>
         </is>
@@ -1915,49 +1950,65 @@
           <t>Java</t>
         </is>
       </c>
-      <c r="I4" t="n">
+      <c r="I4" s="4" t="n">
         <v>3.07</v>
       </c>
-      <c r="J4" s="4" t="inlineStr">
+      <c r="J4" s="5" t="inlineStr">
         <is>
           <t>Bajo</t>
         </is>
       </c>
-      <c r="K4" t="n">
+      <c r="K4" s="4" t="n">
         <v>57.08</v>
       </c>
-      <c r="L4" s="4" t="inlineStr">
+      <c r="L4" s="5" t="inlineStr">
         <is>
           <t>Buena</t>
         </is>
       </c>
-      <c r="M4" t="n">
+      <c r="M4" s="4" t="n">
         <v>9.220000000000001</v>
       </c>
-      <c r="N4" t="n">
+      <c r="N4" s="4" t="n">
         <v>2.75</v>
       </c>
-      <c r="O4" s="4" t="inlineStr">
+      <c r="O4" s="5" t="inlineStr">
         <is>
           <t>Presencia de issues altos</t>
         </is>
       </c>
-      <c r="P4" t="inlineStr"/>
-      <c r="Q4" s="4" t="inlineStr"/>
-      <c r="R4" t="inlineStr"/>
-      <c r="S4" s="4" t="inlineStr"/>
-      <c r="T4" s="5" t="n">
+      <c r="P4" s="6" t="inlineStr">
+        <is>
+          <t>Sin datos</t>
+        </is>
+      </c>
+      <c r="Q4" s="7" t="inlineStr">
+        <is>
+          <t>Sin datos</t>
+        </is>
+      </c>
+      <c r="R4" s="6" t="inlineStr">
+        <is>
+          <t>Sin datos</t>
+        </is>
+      </c>
+      <c r="S4" s="7" t="inlineStr">
+        <is>
+          <t>Sin datos</t>
+        </is>
+      </c>
+      <c r="T4" s="8" t="n">
         <v>1.74375</v>
       </c>
-      <c r="U4" s="4" t="inlineStr">
+      <c r="U4" s="5" t="inlineStr">
         <is>
           <t>Consumo bajo de CPU</t>
         </is>
       </c>
-      <c r="V4" s="5" t="n">
+      <c r="V4" s="8" t="n">
         <v>9.335727109515259</v>
       </c>
-      <c r="W4" s="4" t="inlineStr">
+      <c r="W4" s="5" t="inlineStr">
         <is>
           <t>Consumo bajo de CPU</t>
         </is>
@@ -2004,61 +2055,61 @@
           <t>Kotlin</t>
         </is>
       </c>
-      <c r="I5" t="n">
+      <c r="I5" s="4" t="n">
         <v>1.63</v>
       </c>
-      <c r="J5" s="4" t="inlineStr">
+      <c r="J5" s="5" t="inlineStr">
         <is>
           <t>Bajo</t>
         </is>
       </c>
-      <c r="K5" t="n">
+      <c r="K5" s="4" t="n">
         <v>53.99</v>
       </c>
-      <c r="L5" s="4" t="inlineStr">
+      <c r="L5" s="5" t="inlineStr">
         <is>
           <t>Buena</t>
         </is>
       </c>
-      <c r="M5" t="n">
+      <c r="M5" s="4" t="n">
         <v>104.69</v>
       </c>
-      <c r="N5" t="n">
+      <c r="N5" s="4" t="n">
         <v>1.75</v>
       </c>
-      <c r="O5" s="4" t="inlineStr">
+      <c r="O5" s="5" t="inlineStr">
         <is>
           <t>Predominan issues medios</t>
         </is>
       </c>
-      <c r="P5" t="n">
+      <c r="P5" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="Q5" s="4" t="inlineStr">
+      <c r="Q5" s="5" t="inlineStr">
         <is>
           <t>Muy buen uso de concurrencia</t>
         </is>
       </c>
-      <c r="R5" t="n">
+      <c r="R5" s="4" t="n">
         <v>4.96</v>
       </c>
-      <c r="S5" s="4" t="inlineStr">
+      <c r="S5" s="5" t="inlineStr">
         <is>
           <t>Bajo NLOC/token, ajustada por refinamientos.</t>
         </is>
       </c>
-      <c r="T5" s="5" t="n">
+      <c r="T5" s="8" t="n">
         <v>1.275</v>
       </c>
-      <c r="U5" s="4" t="inlineStr">
+      <c r="U5" s="5" t="inlineStr">
         <is>
           <t>Consumo bajo de CPU</t>
         </is>
       </c>
-      <c r="V5" s="5" t="n">
+      <c r="V5" s="8" t="n">
         <v>16.42728904847397</v>
       </c>
-      <c r="W5" s="4" t="inlineStr">
+      <c r="W5" s="5" t="inlineStr">
         <is>
           <t>Consumo bajo de CPU</t>
         </is>
@@ -2568,7 +2619,7 @@
       <c r="K2" t="n">
         <v>5</v>
       </c>
-      <c r="L2" s="6" t="inlineStr">
+      <c r="L2" s="9" t="inlineStr">
         <is>
           <t>LooseCoupling: 7; UncommentedEmptyMethodBody: 6; LiteralsFirstInComparisons: 6; UnnecessaryImport: 5; SingularField: 1; UnusedPrivateMethod: 1; UseUtilityClass: 1; ClassWithOnlyPrivateConstructorsShouldBeFinal: 1; NonThreadSafeSingleton: 1; MethodNamingConventions: 1</t>
         </is>
@@ -2618,7 +2669,7 @@
       <c r="K3" t="n">
         <v>0</v>
       </c>
-      <c r="L3" s="6" t="inlineStr">
+      <c r="L3" s="9" t="inlineStr">
         <is>
           <t>UncommentedEmptyMethodBody: 6; ClassWithOnlyPrivateConstructorsShouldBeFinal: 2; LooseCoupling: 1</t>
         </is>
@@ -2668,7 +2719,7 @@
       <c r="K4" t="n">
         <v>0</v>
       </c>
-      <c r="L4" s="6" t="inlineStr">
+      <c r="L4" s="9" t="inlineStr">
         <is>
           <t>ControlStatementBraces: 2; UselessQualifiedThis: 1; MethodNamingConventions: 1</t>
         </is>
@@ -2718,7 +2769,7 @@
       <c r="K5" t="n">
         <v>32</v>
       </c>
-      <c r="L5" s="6" t="inlineStr">
+      <c r="L5" s="9" t="inlineStr">
         <is>
           <t>detekt.MagicNumber: 29; detekt.WildcardImport: 16; detekt.FunctionNaming: 13; detekt.MaxLineLength: 3; detekt.LongMethod: 2; detekt.TooGenericExceptionCaught: 2; detekt.SwallowedException: 1; detekt.ReturnCount: 1</t>
         </is>
@@ -3221,7 +3272,7 @@
           <t>Simple</t>
         </is>
       </c>
-      <c r="G2" s="5" t="n">
+      <c r="G2" s="10" t="n">
         <v>1</v>
       </c>
       <c r="H2" t="inlineStr">
@@ -3229,19 +3280,19 @@
           <t>Shake</t>
         </is>
       </c>
-      <c r="I2" s="5" t="n">
+      <c r="I2" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="J2" s="5" t="n">
+      <c r="J2" s="10" t="n">
         <v>0.125</v>
       </c>
-      <c r="K2" s="5" t="n">
+      <c r="K2" s="10" t="n">
         <v>0.125</v>
       </c>
-      <c r="L2" s="5" t="n">
+      <c r="L2" s="10" t="n">
         <v>0.125</v>
       </c>
-      <c r="M2" s="5" t="n">
+      <c r="M2" s="10" t="n">
         <v>0.125</v>
       </c>
       <c r="N2" t="inlineStr">
@@ -3254,22 +3305,22 @@
           <t>Consumo bajo de CPU</t>
         </is>
       </c>
-      <c r="P2" s="7" t="n">
+      <c r="P2" s="11" t="n">
         <v>103</v>
       </c>
-      <c r="Q2" s="7" t="n">
+      <c r="Q2" s="11" t="n">
         <v>111</v>
       </c>
-      <c r="R2" s="7" t="n">
+      <c r="R2" s="11" t="n">
         <v>7792</v>
       </c>
-      <c r="S2" s="7" t="n">
+      <c r="S2" s="11" t="n">
         <v>107</v>
       </c>
-      <c r="T2" s="5" t="n">
+      <c r="T2" s="10" t="n">
         <v>1.373203285420945</v>
       </c>
-      <c r="U2" s="7" t="n">
+      <c r="U2" s="11" t="n">
         <v>111</v>
       </c>
       <c r="V2" t="inlineStr">
@@ -3312,7 +3363,7 @@
           <t>Simple</t>
         </is>
       </c>
-      <c r="G3" s="5" t="n">
+      <c r="G3" s="10" t="n">
         <v>1</v>
       </c>
       <c r="H3" t="inlineStr">
@@ -3320,19 +3371,19 @@
           <t>Shake</t>
         </is>
       </c>
-      <c r="I3" s="5" t="n">
+      <c r="I3" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="J3" s="5" t="n">
+      <c r="J3" s="10" t="n">
         <v>0.125</v>
       </c>
-      <c r="K3" s="5" t="n">
+      <c r="K3" s="10" t="n">
         <v>0.125</v>
       </c>
-      <c r="L3" s="5" t="n">
+      <c r="L3" s="10" t="n">
         <v>0.125</v>
       </c>
-      <c r="M3" s="5" t="n">
+      <c r="M3" s="10" t="n">
         <v>0.125</v>
       </c>
       <c r="N3" t="inlineStr">
@@ -3345,22 +3396,22 @@
           <t>Consumo bajo de CPU</t>
         </is>
       </c>
-      <c r="P3" s="7" t="n">
+      <c r="P3" s="11" t="n">
         <v>104</v>
       </c>
-      <c r="Q3" s="7" t="n">
+      <c r="Q3" s="11" t="n">
         <v>123</v>
       </c>
-      <c r="R3" s="7" t="n">
+      <c r="R3" s="11" t="n">
         <v>7792</v>
       </c>
-      <c r="S3" s="7" t="n">
+      <c r="S3" s="11" t="n">
         <v>113.5</v>
       </c>
-      <c r="T3" s="5" t="n">
+      <c r="T3" s="10" t="n">
         <v>1.456622176591376</v>
       </c>
-      <c r="U3" s="7" t="n">
+      <c r="U3" s="11" t="n">
         <v>123</v>
       </c>
       <c r="V3" t="inlineStr">
@@ -3403,7 +3454,7 @@
           <t>Simple</t>
         </is>
       </c>
-      <c r="G4" s="5" t="n">
+      <c r="G4" s="10" t="n">
         <v>0.8999999999999999</v>
       </c>
       <c r="H4" t="inlineStr">
@@ -3411,19 +3462,19 @@
           <t>leyendo GPS</t>
         </is>
       </c>
-      <c r="I4" s="5" t="n">
+      <c r="I4" s="10" t="n">
         <v>27</v>
       </c>
-      <c r="J4" s="5" t="n">
+      <c r="J4" s="10" t="n">
         <v>0.1125</v>
       </c>
-      <c r="K4" s="5" t="n">
+      <c r="K4" s="10" t="n">
         <v>3.375</v>
       </c>
-      <c r="L4" s="5" t="n">
+      <c r="L4" s="10" t="n">
         <v>1.74375</v>
       </c>
-      <c r="M4" s="5" t="n">
+      <c r="M4" s="10" t="n">
         <v>3.375</v>
       </c>
       <c r="N4" t="inlineStr">
@@ -3436,22 +3487,22 @@
           <t>Consumo bajo de CPU</t>
         </is>
       </c>
-      <c r="P4" s="7" t="n">
+      <c r="P4" s="11" t="n">
         <v>92</v>
       </c>
-      <c r="Q4" s="7" t="n">
+      <c r="Q4" s="11" t="n">
         <v>116</v>
       </c>
-      <c r="R4" s="7" t="n">
+      <c r="R4" s="11" t="n">
         <v>1114</v>
       </c>
-      <c r="S4" s="7" t="n">
+      <c r="S4" s="11" t="n">
         <v>104</v>
       </c>
-      <c r="T4" s="5" t="n">
+      <c r="T4" s="10" t="n">
         <v>9.335727109515259</v>
       </c>
-      <c r="U4" s="7" t="n">
+      <c r="U4" s="11" t="n">
         <v>116</v>
       </c>
       <c r="V4" t="inlineStr">
@@ -3494,7 +3545,7 @@
           <t>Simple</t>
         </is>
       </c>
-      <c r="G5" s="5" t="n">
+      <c r="G5" s="10" t="n">
         <v>2.4</v>
       </c>
       <c r="H5" t="inlineStr">
@@ -3502,19 +3553,19 @@
           <t>leyendo GPS</t>
         </is>
       </c>
-      <c r="I5" s="5" t="n">
+      <c r="I5" s="10" t="n">
         <v>18</v>
       </c>
-      <c r="J5" s="5" t="n">
+      <c r="J5" s="10" t="n">
         <v>0.3</v>
       </c>
-      <c r="K5" s="5" t="n">
+      <c r="K5" s="10" t="n">
         <v>2.25</v>
       </c>
-      <c r="L5" s="5" t="n">
+      <c r="L5" s="10" t="n">
         <v>1.275</v>
       </c>
-      <c r="M5" s="5" t="n">
+      <c r="M5" s="10" t="n">
         <v>2.25</v>
       </c>
       <c r="N5" t="inlineStr">
@@ -3527,22 +3578,22 @@
           <t>Consumo bajo de CPU</t>
         </is>
       </c>
-      <c r="P5" s="7" t="n">
+      <c r="P5" s="11" t="n">
         <v>181</v>
       </c>
-      <c r="Q5" s="7" t="n">
+      <c r="Q5" s="11" t="n">
         <v>185</v>
       </c>
-      <c r="R5" s="7" t="n">
+      <c r="R5" s="11" t="n">
         <v>1114</v>
       </c>
-      <c r="S5" s="7" t="n">
+      <c r="S5" s="11" t="n">
         <v>183</v>
       </c>
-      <c r="T5" s="5" t="n">
+      <c r="T5" s="10" t="n">
         <v>16.42728904847397</v>
       </c>
-      <c r="U5" s="7" t="n">
+      <c r="U5" s="11" t="n">
         <v>185</v>
       </c>
       <c r="V5" t="inlineStr">

</xml_diff>